<commit_message>
content(vacaciones): actualizar el formato de solicitud descargable
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/public/formato-solicitud-vacaciones.xlsx
+++ b/app/public/formato-solicitud-vacaciones.xlsx
@@ -78,10 +78,10 @@
     <t xml:space="preserve">SOLICITUD DE VACACIONES</t>
   </si>
   <si>
-    <t xml:space="preserve">FECHA: 08-Julio-2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE COMPLETO: JUAN PABLO HUIRACOCHA PIEDRA</t>
+    <t xml:space="preserve">FECHA:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOMBRE COMPLETO: </t>
   </si>
   <si>
     <t xml:space="preserve">Por el presente solicito autorización para hacer uso de las vacaciones anuales conforme al siguiente detalle:</t>
@@ -419,13 +419,96 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
+      <xdr:colOff>23040</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>167760</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="1 Imagen"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="74520" y="360"/>
+          <a:ext cx="689400" cy="929520"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:solidFill>
+            <a:srgbClr val="808080"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>246240</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>143280</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>327960</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>43920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="2 Imagen"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3480120" y="143280"/>
+          <a:ext cx="1833840" cy="472320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>74520</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>360</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>23400</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>168120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1 Imagen"/>
+        <xdr:cNvPr id="3" name="1 Imagen"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -452,89 +535,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>246240</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>143280</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>328320</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>44280</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="2 Imagen"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3480120" y="143280"/>
-          <a:ext cx="1834200" cy="472680"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>74520</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>360</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>23760</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>168480</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="1 Imagen"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="74520" y="360"/>
-          <a:ext cx="690120" cy="930240"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:solidFill>
-            <a:srgbClr val="808080"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>322560</xdr:colOff>
       <xdr:row>0</xdr:row>
@@ -542,9 +542,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>661680</xdr:colOff>
+      <xdr:colOff>661320</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>6840</xdr:rowOff>
+      <xdr:rowOff>6480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -558,7 +558,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5071680" y="105480"/>
-          <a:ext cx="1821240" cy="473040"/>
+          <a:ext cx="1820880" cy="472680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>